<commit_message>
bri code and example data updates
modifications to the offshore BRI calculator to reflect B23 benthic index code subcommittee feedback
</commit_message>
<xml_diff>
--- a/SQO dry run/djg test SQO BLOE output summary.xlsx
+++ b/SQO dry run/djg test SQO BLOE output summary.xlsx
@@ -2632,10 +2632,10 @@
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
@@ -2644,7 +2644,7 @@
         <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
         <v>3</v>
@@ -3211,7 +3211,7 @@
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
         <v>2</v>
@@ -5625,7 +5625,7 @@
         <v>2</v>
       </c>
       <c r="G78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H78" t="n">
         <v>2</v>
@@ -8679,7 +8679,7 @@
         <v>42</v>
       </c>
       <c r="F131" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G131" t="n">
         <v>2</v>
@@ -9024,7 +9024,7 @@
         <v>2</v>
       </c>
       <c r="G137" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H137" t="n">
         <v>2</v>
@@ -9316,7 +9316,7 @@
         <v>2</v>
       </c>
       <c r="H142" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I142" t="n">
         <v>3</v>
@@ -9431,7 +9431,7 @@
         <v>2</v>
       </c>
       <c r="G144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H144" t="n">
         <v>4</v>
@@ -9963,7 +9963,7 @@
         <v>2</v>
       </c>
       <c r="H153" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I153" t="n">
         <v>1</v>
@@ -10069,13 +10069,13 @@
         <v>1</v>
       </c>
       <c r="D155" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E155" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="F155" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G155" t="n">
         <v>2</v>
@@ -11780,7 +11780,7 @@
         <v>2</v>
       </c>
       <c r="H184" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I184" t="n">
         <v>3</v>
@@ -12006,7 +12006,7 @@
         <v>26</v>
       </c>
       <c r="F188" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G188" t="n">
         <v>2</v>
@@ -13128,7 +13128,7 @@
         <v>242</v>
       </c>
       <c r="N3" t="n">
-        <v>15.0835121731415</v>
+        <v>15.0836032595324</v>
       </c>
       <c r="O3" t="s">
         <v>20</v>
@@ -13177,7 +13177,7 @@
         <v>242</v>
       </c>
       <c r="N4" t="n">
-        <v>12.1137966502506</v>
+        <v>11.8483309845804</v>
       </c>
       <c r="O4" t="s">
         <v>20</v>
@@ -13226,7 +13226,7 @@
         <v>242</v>
       </c>
       <c r="N5" t="n">
-        <v>13.9117533415191</v>
+        <v>14.9581463094241</v>
       </c>
       <c r="O5" t="s">
         <v>20</v>
@@ -13275,7 +13275,7 @@
         <v>242</v>
       </c>
       <c r="N6" t="n">
-        <v>14.2984796995644</v>
+        <v>14.2996494693632</v>
       </c>
       <c r="O6" t="s">
         <v>20</v>
@@ -13326,7 +13326,7 @@
         <v>242</v>
       </c>
       <c r="N7" t="n">
-        <v>12.5256070876902</v>
+        <v>12.9304384921341</v>
       </c>
       <c r="O7" t="s">
         <v>20</v>
@@ -13375,7 +13375,7 @@
         <v>242</v>
       </c>
       <c r="N8" t="n">
-        <v>8.32587934085862</v>
+        <v>8.6039757528745</v>
       </c>
       <c r="O8" t="s">
         <v>20</v>
@@ -13426,7 +13426,7 @@
         <v>242</v>
       </c>
       <c r="N9" t="n">
-        <v>8.3297123292416</v>
+        <v>8.33034038326227</v>
       </c>
       <c r="O9" t="s">
         <v>20</v>
@@ -13475,7 +13475,7 @@
         <v>242</v>
       </c>
       <c r="N10" t="n">
-        <v>6.89794102129035</v>
+        <v>8.71087727574399</v>
       </c>
       <c r="O10" t="s">
         <v>20</v>
@@ -13524,7 +13524,7 @@
         <v>242</v>
       </c>
       <c r="N11" t="n">
-        <v>7.13429758410547</v>
+        <v>9.7956661477616</v>
       </c>
       <c r="O11" t="s">
         <v>20</v>
@@ -13575,7 +13575,7 @@
         <v>242</v>
       </c>
       <c r="N12" t="n">
-        <v>9.40947000478344</v>
+        <v>9.40985735776787</v>
       </c>
       <c r="O12" t="s">
         <v>20</v>
@@ -13624,7 +13624,7 @@
         <v>242</v>
       </c>
       <c r="N13" t="n">
-        <v>9.02482959811105</v>
+        <v>11.1803875811964</v>
       </c>
       <c r="O13" t="s">
         <v>20</v>
@@ -13673,7 +13673,7 @@
         <v>242</v>
       </c>
       <c r="N14" t="n">
-        <v>13.4161053559657</v>
+        <v>12.3372551759701</v>
       </c>
       <c r="O14" t="s">
         <v>20</v>
@@ -13724,7 +13724,7 @@
         <v>242</v>
       </c>
       <c r="N15" t="n">
-        <v>25.1492945972641</v>
+        <v>25.3364034931308</v>
       </c>
       <c r="O15" t="s">
         <v>20</v>
@@ -13773,7 +13773,7 @@
         <v>242</v>
       </c>
       <c r="N16" t="n">
-        <v>32.7883730254763</v>
+        <v>32.7913138150571</v>
       </c>
       <c r="O16" t="s">
         <v>20</v>
@@ -13822,7 +13822,7 @@
         <v>242</v>
       </c>
       <c r="N17" t="n">
-        <v>36.350454212711</v>
+        <v>33.9697703600652</v>
       </c>
       <c r="O17" t="s">
         <v>20</v>
@@ -13871,7 +13871,7 @@
         <v>242</v>
       </c>
       <c r="N18" t="n">
-        <v>42.407445046611</v>
+        <v>42.4469265154747</v>
       </c>
       <c r="O18" t="s">
         <v>26</v>
@@ -13920,7 +13920,7 @@
         <v>242</v>
       </c>
       <c r="N19" t="n">
-        <v>26.5993771057528</v>
+        <v>26.7370411270221</v>
       </c>
       <c r="O19" t="s">
         <v>20</v>
@@ -13969,7 +13969,7 @@
         <v>242</v>
       </c>
       <c r="N20" t="n">
-        <v>17.8454048383822</v>
+        <v>21.0239865128028</v>
       </c>
       <c r="O20" t="s">
         <v>20</v>
@@ -14018,7 +14018,7 @@
         <v>242</v>
       </c>
       <c r="N21" t="n">
-        <v>32.0488155283212</v>
+        <v>32.2459417423192</v>
       </c>
       <c r="O21" t="s">
         <v>20</v>
@@ -14067,7 +14067,7 @@
         <v>242</v>
       </c>
       <c r="N22" t="n">
-        <v>18.7435227586434</v>
+        <v>21.5044390504018</v>
       </c>
       <c r="O22" t="s">
         <v>20</v>
@@ -14116,7 +14116,7 @@
         <v>242</v>
       </c>
       <c r="N23" t="n">
-        <v>22.8819283339274</v>
+        <v>26.6014204428507</v>
       </c>
       <c r="O23" t="s">
         <v>20</v>
@@ -14165,7 +14165,7 @@
         <v>242</v>
       </c>
       <c r="N24" t="n">
-        <v>34.7453661386161</v>
+        <v>34.4437640570911</v>
       </c>
       <c r="O24" t="s">
         <v>20</v>
@@ -14214,7 +14214,7 @@
         <v>242</v>
       </c>
       <c r="N25" t="n">
-        <v>27.2582157948085</v>
+        <v>27.2610128313953</v>
       </c>
       <c r="O25" t="s">
         <v>20</v>
@@ -14263,7 +14263,7 @@
         <v>242</v>
       </c>
       <c r="N26" t="n">
-        <v>33.3987902247781</v>
+        <v>32.5280831150206</v>
       </c>
       <c r="O26" t="s">
         <v>20</v>
@@ -14312,7 +14312,7 @@
         <v>242</v>
       </c>
       <c r="N27" t="n">
-        <v>44.9967123841401</v>
+        <v>45.0007456972099</v>
       </c>
       <c r="O27" t="s">
         <v>26</v>
@@ -14361,7 +14361,7 @@
         <v>242</v>
       </c>
       <c r="N28" t="n">
-        <v>24.062074209176</v>
+        <v>21.5154834181272</v>
       </c>
       <c r="O28" t="s">
         <v>20</v>
@@ -14410,7 +14410,7 @@
         <v>242</v>
       </c>
       <c r="N29" t="n">
-        <v>42.3141744493955</v>
+        <v>42.0953502737836</v>
       </c>
       <c r="O29" t="s">
         <v>26</v>
@@ -14459,7 +14459,7 @@
         <v>242</v>
       </c>
       <c r="N30" t="n">
-        <v>37.3861784606946</v>
+        <v>37.1629962032474</v>
       </c>
       <c r="O30" t="s">
         <v>20</v>
@@ -14508,7 +14508,7 @@
         <v>242</v>
       </c>
       <c r="N31" t="n">
-        <v>47.2595503811971</v>
+        <v>47.2634331434995</v>
       </c>
       <c r="O31" t="s">
         <v>26</v>
@@ -14557,7 +14557,7 @@
         <v>242</v>
       </c>
       <c r="N32" t="n">
-        <v>44.8646018075336</v>
+        <v>44.8694650103138</v>
       </c>
       <c r="O32" t="s">
         <v>26</v>
@@ -14606,7 +14606,7 @@
         <v>242</v>
       </c>
       <c r="N33" t="n">
-        <v>43.5472187847445</v>
+        <v>43.5512192647488</v>
       </c>
       <c r="O33" t="s">
         <v>26</v>
@@ -14655,7 +14655,7 @@
         <v>242</v>
       </c>
       <c r="N34" t="n">
-        <v>50.968570704329</v>
+        <v>50.550905851502</v>
       </c>
       <c r="O34" t="s">
         <v>42</v>
@@ -14704,7 +14704,7 @@
         <v>242</v>
       </c>
       <c r="N35" t="n">
-        <v>32.243751427066</v>
+        <v>32.1763609084533</v>
       </c>
       <c r="O35" t="s">
         <v>20</v>
@@ -14753,7 +14753,7 @@
         <v>242</v>
       </c>
       <c r="N36" t="n">
-        <v>55.8141715934328</v>
+        <v>57.4863757949222</v>
       </c>
       <c r="O36" t="s">
         <v>42</v>
@@ -14802,7 +14802,7 @@
         <v>242</v>
       </c>
       <c r="N37" t="n">
-        <v>44.2308941636457</v>
+        <v>43.7748376827739</v>
       </c>
       <c r="O37" t="s">
         <v>26</v>
@@ -14851,7 +14851,7 @@
         <v>242</v>
       </c>
       <c r="N38" t="n">
-        <v>39.5021026403308</v>
+        <v>36.0283921978724</v>
       </c>
       <c r="O38" t="s">
         <v>20</v>
@@ -14900,7 +14900,7 @@
         <v>242</v>
       </c>
       <c r="N39" t="n">
-        <v>45.7559329178156</v>
+        <v>46.2484492144239</v>
       </c>
       <c r="O39" t="s">
         <v>26</v>
@@ -14949,7 +14949,7 @@
         <v>242</v>
       </c>
       <c r="N40" t="n">
-        <v>34.480188689579</v>
+        <v>31.1032825790809</v>
       </c>
       <c r="O40" t="s">
         <v>20</v>
@@ -14998,7 +14998,7 @@
         <v>242</v>
       </c>
       <c r="N41" t="n">
-        <v>58.0793879941918</v>
+        <v>58.0832165471716</v>
       </c>
       <c r="O41" t="s">
         <v>42</v>
@@ -15047,7 +15047,7 @@
         <v>242</v>
       </c>
       <c r="N42" t="n">
-        <v>60.9540669023094</v>
+        <v>60.9581009717345</v>
       </c>
       <c r="O42" t="s">
         <v>42</v>
@@ -15096,7 +15096,7 @@
         <v>242</v>
       </c>
       <c r="N43" t="n">
-        <v>32.77020951736</v>
+        <v>32.7738773952884</v>
       </c>
       <c r="O43" t="s">
         <v>20</v>
@@ -15147,7 +15147,7 @@
         <v>242</v>
       </c>
       <c r="N44" t="n">
-        <v>51.8263386730003</v>
+        <v>51.8313447398407</v>
       </c>
       <c r="O44" t="s">
         <v>42</v>
@@ -15198,7 +15198,7 @@
         <v>242</v>
       </c>
       <c r="N45" t="n">
-        <v>60.3555344134806</v>
+        <v>60.3613581672103</v>
       </c>
       <c r="O45" t="s">
         <v>42</v>
@@ -15249,7 +15249,7 @@
         <v>242</v>
       </c>
       <c r="N46" t="n">
-        <v>58.5727683598368</v>
+        <v>58.5769595569426</v>
       </c>
       <c r="O46" t="s">
         <v>42</v>
@@ -15300,7 +15300,7 @@
         <v>242</v>
       </c>
       <c r="N47" t="n">
-        <v>34.6166210092699</v>
+        <v>34.3151407398848</v>
       </c>
       <c r="O47" t="s">
         <v>20</v>
@@ -15351,7 +15351,7 @@
         <v>242</v>
       </c>
       <c r="N48" t="n">
-        <v>34.7825054167021</v>
+        <v>34.4495839027007</v>
       </c>
       <c r="O48" t="s">
         <v>20</v>
@@ -15402,7 +15402,7 @@
         <v>242</v>
       </c>
       <c r="N49" t="n">
-        <v>44.0357694849263</v>
+        <v>44.0394315292482</v>
       </c>
       <c r="O49" t="s">
         <v>26</v>
@@ -15453,7 +15453,7 @@
         <v>242</v>
       </c>
       <c r="N50" t="n">
-        <v>54.2386015325113</v>
+        <v>54.593701476202</v>
       </c>
       <c r="O50" t="s">
         <v>42</v>
@@ -15504,7 +15504,7 @@
         <v>242</v>
       </c>
       <c r="N51" t="n">
-        <v>35.8847263538009</v>
+        <v>35.2484843681082</v>
       </c>
       <c r="O51" t="s">
         <v>20</v>
@@ -15553,7 +15553,7 @@
         <v>242</v>
       </c>
       <c r="N52" t="n">
-        <v>36.2158303405904</v>
+        <v>38.5797223342776</v>
       </c>
       <c r="O52" t="s">
         <v>20</v>
@@ -15602,7 +15602,7 @@
         <v>242</v>
       </c>
       <c r="N53" t="n">
-        <v>33.8497968767349</v>
+        <v>33.7706148627681</v>
       </c>
       <c r="O53" t="s">
         <v>20</v>
@@ -15653,7 +15653,7 @@
         <v>242</v>
       </c>
       <c r="N54" t="n">
-        <v>40.8734564870964</v>
+        <v>41.1151784188755</v>
       </c>
       <c r="O54" t="s">
         <v>26</v>
@@ -15704,7 +15704,7 @@
         <v>242</v>
       </c>
       <c r="N55" t="n">
-        <v>57.6523819222388</v>
+        <v>57.6570724356769</v>
       </c>
       <c r="O55" t="s">
         <v>42</v>
@@ -15753,7 +15753,7 @@
         <v>242</v>
       </c>
       <c r="N56" t="n">
-        <v>51.7196535149094</v>
+        <v>51.7245077283966</v>
       </c>
       <c r="O56" t="s">
         <v>42</v>
@@ -15802,7 +15802,7 @@
         <v>242</v>
       </c>
       <c r="N57" t="n">
-        <v>43.9226507179291</v>
+        <v>44.2645082796971</v>
       </c>
       <c r="O57" t="s">
         <v>26</v>
@@ -15851,7 +15851,7 @@
         <v>242</v>
       </c>
       <c r="N58" t="n">
-        <v>49.8113383496228</v>
+        <v>49.2997982397531</v>
       </c>
       <c r="O58" t="s">
         <v>42</v>
@@ -15900,7 +15900,7 @@
         <v>242</v>
       </c>
       <c r="N59" t="n">
-        <v>36.4369680986238</v>
+        <v>36.161433812764</v>
       </c>
       <c r="O59" t="s">
         <v>20</v>
@@ -15949,7 +15949,7 @@
         <v>242</v>
       </c>
       <c r="N60" t="n">
-        <v>55.111627776202</v>
+        <v>55.1159647984134</v>
       </c>
       <c r="O60" t="s">
         <v>42</v>
@@ -15998,7 +15998,7 @@
         <v>242</v>
       </c>
       <c r="N61" t="n">
-        <v>26.354523282968</v>
+        <v>24.1729318414282</v>
       </c>
       <c r="O61" t="s">
         <v>20</v>
@@ -16047,7 +16047,7 @@
         <v>242</v>
       </c>
       <c r="N62" t="n">
-        <v>46.8685468193033</v>
+        <v>46.8718604742481</v>
       </c>
       <c r="O62" t="s">
         <v>26</v>
@@ -16096,7 +16096,7 @@
         <v>242</v>
       </c>
       <c r="N63" t="n">
-        <v>57.355496186753</v>
+        <v>57.8461293200658</v>
       </c>
       <c r="O63" t="s">
         <v>42</v>
@@ -16145,7 +16145,7 @@
         <v>242</v>
       </c>
       <c r="N64" t="n">
-        <v>61.4518235110778</v>
+        <v>62.6880989195223</v>
       </c>
       <c r="O64" t="s">
         <v>42</v>
@@ -16194,7 +16194,7 @@
         <v>242</v>
       </c>
       <c r="N65" t="n">
-        <v>37.8216472178391</v>
+        <v>37.8755232951499</v>
       </c>
       <c r="O65" t="s">
         <v>20</v>
@@ -16243,7 +16243,7 @@
         <v>242</v>
       </c>
       <c r="N66" t="n">
-        <v>37.8850192357862</v>
+        <v>37.1326695672326</v>
       </c>
       <c r="O66" t="s">
         <v>20</v>
@@ -16292,7 +16292,7 @@
         <v>242</v>
       </c>
       <c r="N67" t="n">
-        <v>33.7332198823278</v>
+        <v>33.640809042433</v>
       </c>
       <c r="O67" t="s">
         <v>20</v>
@@ -16341,7 +16341,7 @@
         <v>242</v>
       </c>
       <c r="N68" t="n">
-        <v>32.6005197925927</v>
+        <v>32.6033919720096</v>
       </c>
       <c r="O68" t="s">
         <v>20</v>
@@ -16390,7 +16390,7 @@
         <v>242</v>
       </c>
       <c r="N69" t="n">
-        <v>48.6600414375087</v>
+        <v>47.9152613664558</v>
       </c>
       <c r="O69" t="s">
         <v>26</v>
@@ -16439,7 +16439,7 @@
         <v>242</v>
       </c>
       <c r="N70" t="n">
-        <v>39.3004160993685</v>
+        <v>37.4402703602602</v>
       </c>
       <c r="O70" t="s">
         <v>20</v>
@@ -16488,7 +16488,7 @@
         <v>242</v>
       </c>
       <c r="N71" t="n">
-        <v>34.2786035957176</v>
+        <v>34.2825329082141</v>
       </c>
       <c r="O71" t="s">
         <v>20</v>
@@ -16537,7 +16537,7 @@
         <v>242</v>
       </c>
       <c r="N72" t="n">
-        <v>31.3191146996047</v>
+        <v>31.2955291311754</v>
       </c>
       <c r="O72" t="s">
         <v>20</v>
@@ -16586,7 +16586,7 @@
         <v>242</v>
       </c>
       <c r="N73" t="n">
-        <v>37.741279233437</v>
+        <v>37.7445607249094</v>
       </c>
       <c r="O73" t="s">
         <v>20</v>
@@ -16635,7 +16635,7 @@
         <v>242</v>
       </c>
       <c r="N74" t="n">
-        <v>35.084232763802</v>
+        <v>33.9284286782615</v>
       </c>
       <c r="O74" t="s">
         <v>20</v>
@@ -16684,7 +16684,7 @@
         <v>242</v>
       </c>
       <c r="N75" t="n">
-        <v>40.569624719579</v>
+        <v>40.3290087302363</v>
       </c>
       <c r="O75" t="s">
         <v>26</v>
@@ -16733,7 +16733,7 @@
         <v>242</v>
       </c>
       <c r="N76" t="n">
-        <v>40.0247396797661</v>
+        <v>40.6459863739937</v>
       </c>
       <c r="O76" t="s">
         <v>26</v>
@@ -16782,7 +16782,7 @@
         <v>242</v>
       </c>
       <c r="N77" t="n">
-        <v>50.7645465283262</v>
+        <v>49.7426953088351</v>
       </c>
       <c r="O77" t="s">
         <v>42</v>
@@ -16831,7 +16831,7 @@
         <v>242</v>
       </c>
       <c r="N78" t="n">
-        <v>53.0902871170182</v>
+        <v>53.5737911776543</v>
       </c>
       <c r="O78" t="s">
         <v>42</v>
@@ -16880,7 +16880,7 @@
         <v>242</v>
       </c>
       <c r="N79" t="n">
-        <v>52.270352748859</v>
+        <v>53.0463318602157</v>
       </c>
       <c r="O79" t="s">
         <v>42</v>
@@ -16929,7 +16929,7 @@
         <v>242</v>
       </c>
       <c r="N80" t="n">
-        <v>48.0404053013533</v>
+        <v>48.6449093133248</v>
       </c>
       <c r="O80" t="s">
         <v>26</v>
@@ -16978,7 +16978,7 @@
         <v>242</v>
       </c>
       <c r="N81" t="n">
-        <v>31.8375</v>
+        <v>31.8428644411</v>
       </c>
       <c r="O81" t="s">
         <v>20</v>
@@ -17027,7 +17027,7 @@
         <v>242</v>
       </c>
       <c r="N82" t="n">
-        <v>58.87137976088</v>
+        <v>58.876742472547</v>
       </c>
       <c r="O82" t="s">
         <v>42</v>
@@ -17076,7 +17076,7 @@
         <v>242</v>
       </c>
       <c r="N83" t="n">
-        <v>57.2921486848901</v>
+        <v>56.2859324071618</v>
       </c>
       <c r="O83" t="s">
         <v>42</v>
@@ -17125,7 +17125,7 @@
         <v>242</v>
       </c>
       <c r="N84" t="n">
-        <v>52.9357739141486</v>
+        <v>52.5511471646297</v>
       </c>
       <c r="O84" t="s">
         <v>42</v>
@@ -17174,7 +17174,7 @@
         <v>242</v>
       </c>
       <c r="N85" t="n">
-        <v>43.1207280752279</v>
+        <v>43.1252283222651</v>
       </c>
       <c r="O85" t="s">
         <v>26</v>
@@ -17225,7 +17225,7 @@
         <v>242</v>
       </c>
       <c r="N86" t="n">
-        <v>23.1899768146899</v>
+        <v>23.1922086297616</v>
       </c>
       <c r="O86" t="s">
         <v>20</v>
@@ -17276,7 +17276,7 @@
         <v>242</v>
       </c>
       <c r="N87" t="n">
-        <v>31.9036720933467</v>
+        <v>31.9065688221437</v>
       </c>
       <c r="O87" t="s">
         <v>20</v>
@@ -17327,7 +17327,7 @@
         <v>242</v>
       </c>
       <c r="N88" t="n">
-        <v>11.2064495439365</v>
+        <v>13.270951521794</v>
       </c>
       <c r="O88" t="s">
         <v>20</v>
@@ -17378,7 +17378,7 @@
         <v>242</v>
       </c>
       <c r="N89" t="n">
-        <v>31.3956585433204</v>
+        <v>31.3979309943615</v>
       </c>
       <c r="O89" t="s">
         <v>20</v>
@@ -17429,7 +17429,7 @@
         <v>242</v>
       </c>
       <c r="N90" t="n">
-        <v>24.5549195255789</v>
+        <v>24.5572040188634</v>
       </c>
       <c r="O90" t="s">
         <v>20</v>
@@ -17478,7 +17478,7 @@
         <v>242</v>
       </c>
       <c r="N91" t="n">
-        <v>12.1942230028456</v>
+        <v>12.1961031744486</v>
       </c>
       <c r="O91" t="s">
         <v>20</v>
@@ -17529,7 +17529,7 @@
         <v>242</v>
       </c>
       <c r="N92" t="n">
-        <v>10.1692205962436</v>
+        <v>10.1705453968361</v>
       </c>
       <c r="O92" t="s">
         <v>20</v>
@@ -17580,7 +17580,7 @@
         <v>242</v>
       </c>
       <c r="N93" t="n">
-        <v>4.86165972694654</v>
+        <v>4.78397879213011</v>
       </c>
       <c r="O93" t="s">
         <v>20</v>
@@ -17631,7 +17631,7 @@
         <v>242</v>
       </c>
       <c r="N94" t="n">
-        <v>16.3825449000804</v>
+        <v>17.9115639941559</v>
       </c>
       <c r="O94" t="s">
         <v>20</v>
@@ -17682,7 +17682,7 @@
         <v>242</v>
       </c>
       <c r="N95" t="n">
-        <v>16.4384752895061</v>
+        <v>17.5891857612011</v>
       </c>
       <c r="O95" t="s">
         <v>20</v>
@@ -17733,7 +17733,7 @@
         <v>242</v>
       </c>
       <c r="N96" t="n">
-        <v>11.6011179093738</v>
+        <v>13.6005680792401</v>
       </c>
       <c r="O96" t="s">
         <v>20</v>
@@ -17782,7 +17782,7 @@
         <v>242</v>
       </c>
       <c r="N97" t="n">
-        <v>7.54409449147013</v>
+        <v>7.66273193633289</v>
       </c>
       <c r="O97" t="s">
         <v>20</v>
@@ -17831,7 +17831,7 @@
         <v>242</v>
       </c>
       <c r="N98" t="n">
-        <v>13.0743521518572</v>
+        <v>13.0752456213904</v>
       </c>
       <c r="O98" t="s">
         <v>20</v>
@@ -17882,7 +17882,7 @@
         <v>242</v>
       </c>
       <c r="N99" t="n">
-        <v>9.84978070834879</v>
+        <v>9.85051761058418</v>
       </c>
       <c r="O99" t="s">
         <v>20</v>
@@ -17933,7 +17933,7 @@
         <v>242</v>
       </c>
       <c r="N100" t="n">
-        <v>34.6138399416805</v>
+        <v>34.6184031988465</v>
       </c>
       <c r="O100" t="s">
         <v>20</v>
@@ -17984,7 +17984,7 @@
         <v>242</v>
       </c>
       <c r="N101" t="n">
-        <v>46.5557479907775</v>
+        <v>46.5596212264505</v>
       </c>
       <c r="O101" t="s">
         <v>26</v>
@@ -18035,7 +18035,7 @@
         <v>242</v>
       </c>
       <c r="N102" t="n">
-        <v>2.14466680647164</v>
+        <v>2.14420429605779</v>
       </c>
       <c r="O102" t="s">
         <v>20</v>
@@ -18086,7 +18086,7 @@
         <v>242</v>
       </c>
       <c r="N103" t="n">
-        <v>1.98262451009629</v>
+        <v>1.32081676762569</v>
       </c>
       <c r="O103" t="s">
         <v>20</v>
@@ -18135,7 +18135,7 @@
         <v>242</v>
       </c>
       <c r="N104" t="n">
-        <v>11.6191894602328</v>
+        <v>11.6202773536615</v>
       </c>
       <c r="O104" t="s">
         <v>20</v>
@@ -18186,7 +18186,7 @@
         <v>242</v>
       </c>
       <c r="N105" t="n">
-        <v>10.3387676701061</v>
+        <v>11.6383482184709</v>
       </c>
       <c r="O105" t="s">
         <v>20</v>
@@ -18235,7 +18235,7 @@
         <v>242</v>
       </c>
       <c r="N106" t="n">
-        <v>9.38646772240299</v>
+        <v>9.38811959642256</v>
       </c>
       <c r="O106" t="s">
         <v>20</v>
@@ -18286,7 +18286,7 @@
         <v>242</v>
       </c>
       <c r="N107" t="n">
-        <v>4.80542773699556</v>
+        <v>8.16961064333156</v>
       </c>
       <c r="O107" t="s">
         <v>20</v>
@@ -18337,7 +18337,7 @@
         <v>242</v>
       </c>
       <c r="N108" t="n">
-        <v>10.1747537747187</v>
+        <v>12.1040470010412</v>
       </c>
       <c r="O108" t="s">
         <v>20</v>
@@ -18386,7 +18386,7 @@
         <v>242</v>
       </c>
       <c r="N109" t="n">
-        <v>31.1211257581424</v>
+        <v>30.6644086042866</v>
       </c>
       <c r="O109" t="s">
         <v>20</v>
@@ -18435,7 +18435,7 @@
         <v>242</v>
       </c>
       <c r="N110" t="n">
-        <v>47.1897965528831</v>
+        <v>46.6256547683002</v>
       </c>
       <c r="O110" t="s">
         <v>26</v>
@@ -18484,7 +18484,7 @@
         <v>242</v>
       </c>
       <c r="N111" t="n">
-        <v>36.1227151646562</v>
+        <v>35.8360658033654</v>
       </c>
       <c r="O111" t="s">
         <v>20</v>
@@ -18533,7 +18533,7 @@
         <v>242</v>
       </c>
       <c r="N112" t="n">
-        <v>42.5421191400731</v>
+        <v>44.7565103451307</v>
       </c>
       <c r="O112" t="s">
         <v>26</v>
@@ -18582,7 +18582,7 @@
         <v>242</v>
       </c>
       <c r="N113" t="n">
-        <v>43.8461235237061</v>
+        <v>42.7624117274131</v>
       </c>
       <c r="O113" t="s">
         <v>26</v>
@@ -18631,7 +18631,7 @@
         <v>242</v>
       </c>
       <c r="N114" t="n">
-        <v>27.3189987855729</v>
+        <v>27.5299886947659</v>
       </c>
       <c r="O114" t="s">
         <v>20</v>
@@ -18680,7 +18680,7 @@
         <v>242</v>
       </c>
       <c r="N115" t="n">
-        <v>21.5284937020595</v>
+        <v>20.6405849047233</v>
       </c>
       <c r="O115" t="s">
         <v>20</v>
@@ -18729,7 +18729,7 @@
         <v>242</v>
       </c>
       <c r="N116" t="n">
-        <v>48.2853416352102</v>
+        <v>47.4585847681724</v>
       </c>
       <c r="O116" t="s">
         <v>26</v>
@@ -18778,7 +18778,7 @@
         <v>242</v>
       </c>
       <c r="N117" t="n">
-        <v>24.6906614267598</v>
+        <v>23.8355136573165</v>
       </c>
       <c r="O117" t="s">
         <v>20</v>
@@ -18827,7 +18827,7 @@
         <v>242</v>
       </c>
       <c r="N118" t="n">
-        <v>36.2570045434227</v>
+        <v>37.7801970738236</v>
       </c>
       <c r="O118" t="s">
         <v>20</v>
@@ -18876,7 +18876,7 @@
         <v>242</v>
       </c>
       <c r="N119" t="n">
-        <v>21.4965155439</v>
+        <v>21.4978404899989</v>
       </c>
       <c r="O119" t="s">
         <v>20</v>
@@ -18925,7 +18925,7 @@
         <v>242</v>
       </c>
       <c r="N120" t="n">
-        <v>46.1964999441301</v>
+        <v>46.2000741490114</v>
       </c>
       <c r="O120" t="s">
         <v>26</v>
@@ -18974,7 +18974,7 @@
         <v>242</v>
       </c>
       <c r="N121" t="n">
-        <v>66.6622743885865</v>
+        <v>66.6661098221637</v>
       </c>
       <c r="O121" t="s">
         <v>42</v>
@@ -19023,7 +19023,7 @@
         <v>242</v>
       </c>
       <c r="N122" t="n">
-        <v>57.0222130349308</v>
+        <v>57.026510365107</v>
       </c>
       <c r="O122" t="s">
         <v>42</v>
@@ -19072,7 +19072,7 @@
         <v>242</v>
       </c>
       <c r="N123" t="n">
-        <v>47.1882343413431</v>
+        <v>48.3906204338871</v>
       </c>
       <c r="O123" t="s">
         <v>26</v>
@@ -19121,7 +19121,7 @@
         <v>242</v>
       </c>
       <c r="N124" t="n">
-        <v>47.8482770760628</v>
+        <v>47.852521720281</v>
       </c>
       <c r="O124" t="s">
         <v>26</v>
@@ -19170,7 +19170,7 @@
         <v>242</v>
       </c>
       <c r="N125" t="n">
-        <v>64.0805893132035</v>
+        <v>64.0849572302475</v>
       </c>
       <c r="O125" t="s">
         <v>42</v>
@@ -19219,7 +19219,7 @@
         <v>242</v>
       </c>
       <c r="N126" t="n">
-        <v>38.425469626862</v>
+        <v>38.429474379491</v>
       </c>
       <c r="O126" t="s">
         <v>20</v>
@@ -19268,7 +19268,7 @@
         <v>242</v>
       </c>
       <c r="N127" t="n">
-        <v>41.3274729396881</v>
+        <v>41.3310423144838</v>
       </c>
       <c r="O127" t="s">
         <v>26</v>
@@ -19317,7 +19317,7 @@
         <v>242</v>
       </c>
       <c r="N128" t="n">
-        <v>44.2985559045416</v>
+        <v>44.3034349249428</v>
       </c>
       <c r="O128" t="s">
         <v>26</v>
@@ -19366,7 +19366,7 @@
         <v>242</v>
       </c>
       <c r="N129" t="n">
-        <v>40.4725794243005</v>
+        <v>40.8727281383874</v>
       </c>
       <c r="O129" t="s">
         <v>26</v>
@@ -19415,7 +19415,7 @@
         <v>242</v>
       </c>
       <c r="N130" t="n">
-        <v>40.3502360309018</v>
+        <v>41.9807099288077</v>
       </c>
       <c r="O130" t="s">
         <v>26</v>
@@ -19464,7 +19464,7 @@
         <v>242</v>
       </c>
       <c r="N131" t="n">
-        <v>44.6572184297854</v>
+        <v>44.6615340709059</v>
       </c>
       <c r="O131" t="s">
         <v>26</v>
@@ -19513,7 +19513,7 @@
         <v>242</v>
       </c>
       <c r="N132" t="n">
-        <v>45.3330176218466</v>
+        <v>45.3376123556685</v>
       </c>
       <c r="O132" t="s">
         <v>26</v>
@@ -19562,13 +19562,13 @@
         <v>242</v>
       </c>
       <c r="N133" t="n">
-        <v>49.8333351317402</v>
+        <v>48.9228614521441</v>
       </c>
       <c r="O133" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="P133" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q133"/>
     </row>
@@ -19611,7 +19611,7 @@
         <v>242</v>
       </c>
       <c r="N134" t="n">
-        <v>52.2772886396889</v>
+        <v>51.4091444274823</v>
       </c>
       <c r="O134" t="s">
         <v>42</v>
@@ -19660,7 +19660,7 @@
         <v>242</v>
       </c>
       <c r="N135" t="n">
-        <v>49.5920964985622</v>
+        <v>49.597075379376</v>
       </c>
       <c r="O135" t="s">
         <v>42</v>
@@ -19709,7 +19709,7 @@
         <v>242</v>
       </c>
       <c r="N136" t="n">
-        <v>49.8294054830651</v>
+        <v>49.8322908697209</v>
       </c>
       <c r="O136" t="s">
         <v>42</v>
@@ -19758,7 +19758,7 @@
         <v>242</v>
       </c>
       <c r="N137" t="n">
-        <v>42.7972122978928</v>
+        <v>42.8005761488192</v>
       </c>
       <c r="O137" t="s">
         <v>26</v>
@@ -19807,7 +19807,7 @@
         <v>242</v>
       </c>
       <c r="N138" t="n">
-        <v>40.8134536927987</v>
+        <v>42.314685818171</v>
       </c>
       <c r="O138" t="s">
         <v>26</v>
@@ -19856,7 +19856,7 @@
         <v>242</v>
       </c>
       <c r="N139" t="n">
-        <v>42.9428751180818</v>
+        <v>42.4230650178746</v>
       </c>
       <c r="O139" t="s">
         <v>26</v>
@@ -19905,7 +19905,7 @@
         <v>242</v>
       </c>
       <c r="N140" t="n">
-        <v>42.5655223220909</v>
+        <v>44.7006950436784</v>
       </c>
       <c r="O140" t="s">
         <v>26</v>
@@ -19954,7 +19954,7 @@
         <v>242</v>
       </c>
       <c r="N141" t="n">
-        <v>41.7342042409386</v>
+        <v>41.7753303847744</v>
       </c>
       <c r="O141" t="s">
         <v>26</v>
@@ -20005,7 +20005,7 @@
         <v>242</v>
       </c>
       <c r="N142" t="n">
-        <v>38.3068553435736</v>
+        <v>38.311041234604</v>
       </c>
       <c r="O142" t="s">
         <v>20</v>
@@ -20056,7 +20056,7 @@
         <v>242</v>
       </c>
       <c r="N143" t="n">
-        <v>63.4756400968901</v>
+        <v>68.1876518214113</v>
       </c>
       <c r="O143" t="s">
         <v>42</v>
@@ -20107,7 +20107,7 @@
         <v>242</v>
       </c>
       <c r="N144" t="n">
-        <v>44.9715080857073</v>
+        <v>46.0604562850646</v>
       </c>
       <c r="O144" t="s">
         <v>26</v>
@@ -20158,7 +20158,7 @@
         <v>242</v>
       </c>
       <c r="N145" t="n">
-        <v>35.7036831742656</v>
+        <v>35.6278547478465</v>
       </c>
       <c r="O145" t="s">
         <v>20</v>
@@ -20207,7 +20207,7 @@
         <v>242</v>
       </c>
       <c r="N146" t="n">
-        <v>46.0046484336742</v>
+        <v>47.2565507810849</v>
       </c>
       <c r="O146" t="s">
         <v>26</v>
@@ -20258,7 +20258,7 @@
         <v>242</v>
       </c>
       <c r="N147" t="n">
-        <v>51.9132617715786</v>
+        <v>51.9173492799867</v>
       </c>
       <c r="O147" t="s">
         <v>42</v>
@@ -20309,7 +20309,7 @@
         <v>242</v>
       </c>
       <c r="N148" t="n">
-        <v>63.0742143131437</v>
+        <v>63.0776182048867</v>
       </c>
       <c r="O148" t="s">
         <v>42</v>
@@ -20360,7 +20360,7 @@
         <v>242</v>
       </c>
       <c r="N149" t="n">
-        <v>46.9510047562081</v>
+        <v>45.8220839569622</v>
       </c>
       <c r="O149" t="s">
         <v>26</v>
@@ -20411,7 +20411,7 @@
         <v>242</v>
       </c>
       <c r="N150" t="n">
-        <v>59.6198818020546</v>
+        <v>59.6532996938498</v>
       </c>
       <c r="O150" t="s">
         <v>42</v>
@@ -20462,7 +20462,7 @@
         <v>242</v>
       </c>
       <c r="N151" t="n">
-        <v>48.2981999328139</v>
+        <v>46.969130247006</v>
       </c>
       <c r="O151" t="s">
         <v>26</v>
@@ -20513,7 +20513,7 @@
         <v>242</v>
       </c>
       <c r="N152" t="n">
-        <v>42.6542539120847</v>
+        <v>42.9836210661531</v>
       </c>
       <c r="O152" t="s">
         <v>26</v>
@@ -20564,7 +20564,7 @@
         <v>242</v>
       </c>
       <c r="N153" t="n">
-        <v>43.3427236763665</v>
+        <v>41.1157080768444</v>
       </c>
       <c r="O153" t="s">
         <v>26</v>
@@ -20615,7 +20615,7 @@
         <v>242</v>
       </c>
       <c r="N154" t="n">
-        <v>44.0802014732414</v>
+        <v>41.6660057447824</v>
       </c>
       <c r="O154" t="s">
         <v>26</v>
@@ -20666,7 +20666,7 @@
         <v>242</v>
       </c>
       <c r="N155" t="n">
-        <v>48.5484662475755</v>
+        <v>47.6826464123334</v>
       </c>
       <c r="O155" t="s">
         <v>26</v>
@@ -20717,7 +20717,7 @@
         <v>242</v>
       </c>
       <c r="N156" t="n">
-        <v>45.2339532445515</v>
+        <v>44.2227130443011</v>
       </c>
       <c r="O156" t="s">
         <v>26</v>
@@ -20768,13 +20768,13 @@
         <v>242</v>
       </c>
       <c r="N157" t="n">
-        <v>43.1894911623646</v>
+        <v>50.3200075560917</v>
       </c>
       <c r="O157" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="P157" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q157"/>
     </row>
@@ -20819,7 +20819,7 @@
         <v>242</v>
       </c>
       <c r="N158" t="n">
-        <v>54.3283280945605</v>
+        <v>54.3331519508221</v>
       </c>
       <c r="O158" t="s">
         <v>42</v>
@@ -20870,7 +20870,7 @@
         <v>242</v>
       </c>
       <c r="N159" t="n">
-        <v>70.1149135277061</v>
+        <v>70.121401370688</v>
       </c>
       <c r="O159" t="s">
         <v>42</v>
@@ -20921,7 +20921,7 @@
         <v>242</v>
       </c>
       <c r="N160" t="n">
-        <v>66.1471478991895</v>
+        <v>63.4361802885292</v>
       </c>
       <c r="O160" t="s">
         <v>42</v>
@@ -20972,7 +20972,7 @@
         <v>242</v>
       </c>
       <c r="N161" t="n">
-        <v>42.4352947696759</v>
+        <v>42.4398982678953</v>
       </c>
       <c r="O161" t="s">
         <v>26</v>
@@ -21023,7 +21023,7 @@
         <v>242</v>
       </c>
       <c r="N162" t="n">
-        <v>68.3605870855828</v>
+        <v>64.1733843858322</v>
       </c>
       <c r="O162" t="s">
         <v>42</v>
@@ -21074,7 +21074,7 @@
         <v>242</v>
       </c>
       <c r="N163" t="n">
-        <v>44.9140114323532</v>
+        <v>47.5424121211345</v>
       </c>
       <c r="O163" t="s">
         <v>26</v>
@@ -21125,7 +21125,7 @@
         <v>242</v>
       </c>
       <c r="N164" t="n">
-        <v>53.3093343490612</v>
+        <v>51.1126212670072</v>
       </c>
       <c r="O164" t="s">
         <v>42</v>
@@ -21176,7 +21176,7 @@
         <v>242</v>
       </c>
       <c r="N165" t="n">
-        <v>51.6833585712822</v>
+        <v>49.4444629115014</v>
       </c>
       <c r="O165" t="s">
         <v>42</v>
@@ -21227,7 +21227,7 @@
         <v>242</v>
       </c>
       <c r="N166" t="n">
-        <v>50.4274547413038</v>
+        <v>50.4339111615517</v>
       </c>
       <c r="O166" t="s">
         <v>42</v>
@@ -21278,7 +21278,7 @@
         <v>242</v>
       </c>
       <c r="N167" t="n">
-        <v>68.4830632118997</v>
+        <v>67.6395071626007</v>
       </c>
       <c r="O167" t="s">
         <v>42</v>
@@ -21329,7 +21329,7 @@
         <v>242</v>
       </c>
       <c r="N168" t="n">
-        <v>47.473094180015</v>
+        <v>47.4786861844209</v>
       </c>
       <c r="O168" t="s">
         <v>26</v>
@@ -21378,7 +21378,7 @@
         <v>242</v>
       </c>
       <c r="N169" t="n">
-        <v>43.9115161761981</v>
+        <v>43.9143318015873</v>
       </c>
       <c r="O169" t="s">
         <v>26</v>
@@ -21427,7 +21427,7 @@
         <v>242</v>
       </c>
       <c r="N170" t="n">
-        <v>43.8035949993957</v>
+        <v>43.807472742447</v>
       </c>
       <c r="O170" t="s">
         <v>26</v>
@@ -21476,7 +21476,7 @@
         <v>242</v>
       </c>
       <c r="N171" t="n">
-        <v>60.0973152227697</v>
+        <v>60.102476593241</v>
       </c>
       <c r="O171" t="s">
         <v>42</v>
@@ -21525,7 +21525,7 @@
         <v>242</v>
       </c>
       <c r="N172" t="n">
-        <v>44.5089404393813</v>
+        <v>44.5129157272546</v>
       </c>
       <c r="O172" t="s">
         <v>26</v>
@@ -21576,7 +21576,7 @@
         <v>242</v>
       </c>
       <c r="N173" t="n">
-        <v>45.8726229655959</v>
+        <v>45.1214524227251</v>
       </c>
       <c r="O173" t="s">
         <v>26</v>
@@ -21674,7 +21674,7 @@
         <v>242</v>
       </c>
       <c r="N175" t="n">
-        <v>80.5555032440556</v>
+        <v>79.1787504698617</v>
       </c>
       <c r="O175" t="s">
         <v>38</v>
@@ -21725,7 +21725,7 @@
         <v>242</v>
       </c>
       <c r="N176" t="n">
-        <v>69.95</v>
+        <v>69.9587992</v>
       </c>
       <c r="O176" t="s">
         <v>42</v>
@@ -21776,7 +21776,7 @@
         <v>242</v>
       </c>
       <c r="N177" t="n">
-        <v>31.37</v>
+        <v>31.379525007</v>
       </c>
       <c r="O177" t="s">
         <v>20</v>
@@ -21827,7 +21827,7 @@
         <v>242</v>
       </c>
       <c r="N178" t="n">
-        <v>65.6001183025116</v>
+        <v>64.0567320807063</v>
       </c>
       <c r="O178" t="s">
         <v>42</v>
@@ -21878,7 +21878,7 @@
         <v>242</v>
       </c>
       <c r="N179" t="n">
-        <v>100.914152888188</v>
+        <v>103.575012595292</v>
       </c>
       <c r="O179" t="s">
         <v>38</v>
@@ -21929,7 +21929,7 @@
         <v>242</v>
       </c>
       <c r="N180" t="n">
-        <v>100.846655654698</v>
+        <v>103.376414891309</v>
       </c>
       <c r="O180" t="s">
         <v>38</v>
@@ -21980,7 +21980,7 @@
         <v>242</v>
       </c>
       <c r="N181" t="n">
-        <v>92.4425500632061</v>
+        <v>90.7419499720894</v>
       </c>
       <c r="O181" t="s">
         <v>38</v>
@@ -22031,7 +22031,7 @@
         <v>242</v>
       </c>
       <c r="N182" t="n">
-        <v>62.9939853131011</v>
+        <v>60.5341403489081</v>
       </c>
       <c r="O182" t="s">
         <v>42</v>
@@ -22082,7 +22082,7 @@
         <v>242</v>
       </c>
       <c r="N183" t="n">
-        <v>80.2993623979004</v>
+        <v>82.9432288876675</v>
       </c>
       <c r="O183" t="s">
         <v>38</v>
@@ -22131,7 +22131,7 @@
         <v>242</v>
       </c>
       <c r="N184" t="n">
-        <v>62.9996282426913</v>
+        <v>59.773849666236</v>
       </c>
       <c r="O184" t="s">
         <v>42</v>
@@ -22182,7 +22182,7 @@
         <v>242</v>
       </c>
       <c r="N185" t="n">
-        <v>46.2481291843476</v>
+        <v>41.7268992562071</v>
       </c>
       <c r="O185" t="s">
         <v>26</v>
@@ -22233,7 +22233,7 @@
         <v>242</v>
       </c>
       <c r="N186" t="n">
-        <v>47.348539207356</v>
+        <v>43.764771987482</v>
       </c>
       <c r="O186" t="s">
         <v>26</v>
@@ -22284,7 +22284,7 @@
         <v>242</v>
       </c>
       <c r="N187" t="n">
-        <v>67.1334226495279</v>
+        <v>67.1375967349711</v>
       </c>
       <c r="O187" t="s">
         <v>42</v>
@@ -22333,7 +22333,7 @@
         <v>242</v>
       </c>
       <c r="N188" t="n">
-        <v>14.5376272087859</v>
+        <v>15.0973837903592</v>
       </c>
       <c r="O188" t="s">
         <v>20</v>
@@ -22382,7 +22382,7 @@
         <v>242</v>
       </c>
       <c r="N189" t="n">
-        <v>12.5680670664863</v>
+        <v>12.5698046426121</v>
       </c>
       <c r="O189" t="s">
         <v>20</v>
@@ -22431,13 +22431,13 @@
         <v>242</v>
       </c>
       <c r="N190" t="n">
-        <v>40.8019214988018</v>
+        <v>39.3743639877656</v>
       </c>
       <c r="O190" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="P190" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q190"/>
     </row>
@@ -22480,7 +22480,7 @@
         <v>242</v>
       </c>
       <c r="N191" t="n">
-        <v>29.1883826253006</v>
+        <v>28.701506477696</v>
       </c>
       <c r="O191" t="s">
         <v>20</v>
@@ -22529,7 +22529,7 @@
         <v>242</v>
       </c>
       <c r="N192" t="n">
-        <v>42.8291806733234</v>
+        <v>41.7027444687709</v>
       </c>
       <c r="O192" t="s">
         <v>26</v>
@@ -22578,7 +22578,7 @@
         <v>242</v>
       </c>
       <c r="N193" t="n">
-        <v>69.95</v>
+        <v>69.9587992</v>
       </c>
       <c r="O193" t="s">
         <v>42</v>
@@ -22629,7 +22629,7 @@
         <v>242</v>
       </c>
       <c r="N194" t="n">
-        <v>77.6361392954012</v>
+        <v>77.6408201529544</v>
       </c>
       <c r="O194" t="s">
         <v>38</v>
@@ -22680,7 +22680,7 @@
         <v>242</v>
       </c>
       <c r="N195" t="n">
-        <v>32.8584426583852</v>
+        <v>33.1764519722665</v>
       </c>
       <c r="O195" t="s">
         <v>20</v>
@@ -22731,7 +22731,7 @@
         <v>242</v>
       </c>
       <c r="N196" t="n">
-        <v>62.8240924171001</v>
+        <v>64.9895164357706</v>
       </c>
       <c r="O196" t="s">
         <v>42</v>
@@ -22876,7 +22876,7 @@
         <v>242</v>
       </c>
       <c r="N199" t="n">
-        <v>77.367859953028</v>
+        <v>77.3725439867089</v>
       </c>
       <c r="O199" t="s">
         <v>38</v>
@@ -22927,7 +22927,7 @@
         <v>242</v>
       </c>
       <c r="N200" t="n">
-        <v>69.95</v>
+        <v>69.9587992</v>
       </c>
       <c r="O200" t="s">
         <v>42</v>
@@ -23025,7 +23025,7 @@
         <v>242</v>
       </c>
       <c r="N202" t="n">
-        <v>49.5749956358063</v>
+        <v>49.5791316120116</v>
       </c>
       <c r="O202" t="s">
         <v>42</v>
@@ -23076,7 +23076,7 @@
         <v>242</v>
       </c>
       <c r="N203" t="n">
-        <v>73.0302715390466</v>
+        <v>73.0362981218374</v>
       </c>
       <c r="O203" t="s">
         <v>42</v>
@@ -23127,7 +23127,7 @@
         <v>242</v>
       </c>
       <c r="N204" t="n">
-        <v>56.484274471388</v>
+        <v>55.1331427182267</v>
       </c>
       <c r="O204" t="s">
         <v>42</v>
@@ -25084,13 +25084,13 @@
         <v>245</v>
       </c>
       <c r="N38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O38" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="P38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q38" t="s">
         <v>246</v>
@@ -27246,13 +27246,13 @@
         <v>245</v>
       </c>
       <c r="N80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O80" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="P80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q80" t="s">
         <v>246</v>
@@ -30291,13 +30291,13 @@
         <v>245</v>
       </c>
       <c r="N139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O139" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="P139" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q139" t="s">
         <v>246</v>
@@ -30656,13 +30656,13 @@
         <v>245</v>
       </c>
       <c r="N146" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O146" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="P146" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q146" t="s">
         <v>246</v>
@@ -34184,7 +34184,7 @@
         <v>247</v>
       </c>
       <c r="N9" t="n">
-        <v>0.189321402691411</v>
+        <v>0.191475136188428</v>
       </c>
       <c r="O9" t="s">
         <v>26</v>
@@ -34286,7 +34286,7 @@
         <v>247</v>
       </c>
       <c r="N11" t="n">
-        <v>0.178379829095246</v>
+        <v>0.180533562592263</v>
       </c>
       <c r="O11" t="s">
         <v>26</v>
@@ -34390,7 +34390,7 @@
         <v>247</v>
       </c>
       <c r="N13" t="n">
-        <v>0.198906514411919</v>
+        <v>0.201060247908936</v>
       </c>
       <c r="O13" t="s">
         <v>26</v>
@@ -34441,7 +34441,7 @@
         <v>247</v>
       </c>
       <c r="N14" t="n">
-        <v>0.253842949341174</v>
+        <v>0.255996682838191</v>
       </c>
       <c r="O14" t="s">
         <v>26</v>
@@ -34596,7 +34596,7 @@
         <v>247</v>
       </c>
       <c r="N17" t="n">
-        <v>0.259277493457965</v>
+        <v>0.268846598457712</v>
       </c>
       <c r="O17" t="s">
         <v>26</v>
@@ -34647,7 +34647,7 @@
         <v>247</v>
       </c>
       <c r="N18" t="n">
-        <v>0.22485494504881</v>
+        <v>0.222701211551793</v>
       </c>
       <c r="O18" t="s">
         <v>26</v>
@@ -34698,7 +34698,7 @@
         <v>247</v>
       </c>
       <c r="N19" t="n">
-        <v>0.145856769427758</v>
+        <v>0.1556254892178</v>
       </c>
       <c r="O19" t="s">
         <v>42</v>
@@ -34800,7 +34800,7 @@
         <v>247</v>
       </c>
       <c r="N21" t="n">
-        <v>0.759605072469519</v>
+        <v>0.767083414916195</v>
       </c>
       <c r="O21" t="s">
         <v>20</v>
@@ -34851,7 +34851,7 @@
         <v>247</v>
       </c>
       <c r="N22" t="n">
-        <v>0.771634163538059</v>
+        <v>0.781203268537805</v>
       </c>
       <c r="O22" t="s">
         <v>20</v>
@@ -35157,13 +35157,13 @@
         <v>247</v>
       </c>
       <c r="N28" t="n">
-        <v>0.155302054444533</v>
+        <v>0.164997101332174</v>
       </c>
       <c r="O28" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="P28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q28" t="s">
         <v>246</v>
@@ -35514,7 +35514,7 @@
         <v>247</v>
       </c>
       <c r="N35" t="n">
-        <v>0.196074034540926</v>
+        <v>0.198227768037943</v>
       </c>
       <c r="O35" t="s">
         <v>26</v>
@@ -35565,7 +35565,7 @@
         <v>247</v>
       </c>
       <c r="N36" t="n">
-        <v>0.0712752423970888</v>
+        <v>0.0691215089000718</v>
       </c>
       <c r="O36" t="s">
         <v>38</v>
@@ -35718,7 +35718,7 @@
         <v>247</v>
       </c>
       <c r="N39" t="n">
-        <v>0.187011088779152</v>
+        <v>0.184857355282135</v>
       </c>
       <c r="O39" t="s">
         <v>26</v>
@@ -35922,7 +35922,7 @@
         <v>247</v>
       </c>
       <c r="N43" t="n">
-        <v>0.366734095729723</v>
+        <v>0.376271715257496</v>
       </c>
       <c r="O43" t="s">
         <v>20</v>
@@ -36240,7 +36240,7 @@
         <v>247</v>
       </c>
       <c r="N49" t="n">
-        <v>0.241347881307264</v>
+        <v>0.260580547722678</v>
       </c>
       <c r="O49" t="s">
         <v>26</v>
@@ -36293,7 +36293,7 @@
         <v>247</v>
       </c>
       <c r="N50" t="n">
-        <v>0.160277512900468</v>
+        <v>0.179415722899961</v>
       </c>
       <c r="O50" t="s">
         <v>26</v>
@@ -36397,7 +36397,7 @@
         <v>247</v>
       </c>
       <c r="N52" t="n">
-        <v>0.430880281817545</v>
+        <v>0.438495268110569</v>
       </c>
       <c r="O52" t="s">
         <v>20</v>
@@ -36448,7 +36448,7 @@
         <v>247</v>
       </c>
       <c r="N53" t="n">
-        <v>0.423380536643283</v>
+        <v>0.43294964164303</v>
       </c>
       <c r="O53" t="s">
         <v>20</v>
@@ -36501,7 +36501,7 @@
         <v>247</v>
       </c>
       <c r="N54" t="n">
-        <v>0.33026081993043</v>
+        <v>0.33830590087263</v>
       </c>
       <c r="O54" t="s">
         <v>20</v>
@@ -36605,7 +36605,7 @@
         <v>247</v>
       </c>
       <c r="N56" t="n">
-        <v>0.0690936126810361</v>
+        <v>0.0786312322088091</v>
       </c>
       <c r="O56" t="s">
         <v>38</v>
@@ -36656,7 +36656,7 @@
         <v>247</v>
       </c>
       <c r="N57" t="n">
-        <v>0.168308278191142</v>
+        <v>0.190626520859961</v>
       </c>
       <c r="O57" t="s">
         <v>26</v>
@@ -36758,7 +36758,7 @@
         <v>247</v>
       </c>
       <c r="N59" t="n">
-        <v>0.396805551224153</v>
+        <v>0.416573470663116</v>
       </c>
       <c r="O59" t="s">
         <v>20</v>
@@ -36962,7 +36962,7 @@
         <v>247</v>
       </c>
       <c r="N63" t="n">
-        <v>0.0724219154935461</v>
+        <v>0.070268181996529</v>
       </c>
       <c r="O63" t="s">
         <v>38</v>
@@ -37013,7 +37013,7 @@
         <v>247</v>
       </c>
       <c r="N64" t="n">
-        <v>0.0427476056192509</v>
+        <v>0.0405938721222338</v>
       </c>
       <c r="O64" t="s">
         <v>38</v>
@@ -37064,7 +37064,7 @@
         <v>247</v>
       </c>
       <c r="N65" t="n">
-        <v>0.286334683939384</v>
+        <v>0.284180950442367</v>
       </c>
       <c r="O65" t="s">
         <v>20</v>
@@ -37217,7 +37217,7 @@
         <v>247</v>
       </c>
       <c r="N68" t="n">
-        <v>0.0697522451384839</v>
+        <v>0.0740597121325181</v>
       </c>
       <c r="O68" t="s">
         <v>38</v>
@@ -37421,7 +37421,7 @@
         <v>247</v>
       </c>
       <c r="N72" t="n">
-        <v>0.387777720632359</v>
+        <v>0.39747276752</v>
       </c>
       <c r="O72" t="s">
         <v>20</v>
@@ -37523,7 +37523,7 @@
         <v>247</v>
       </c>
       <c r="N74" t="n">
-        <v>0.643747857559407</v>
+        <v>0.653568846334942</v>
       </c>
       <c r="O74" t="s">
         <v>20</v>
@@ -37625,7 +37625,7 @@
         <v>247</v>
       </c>
       <c r="N76" t="n">
-        <v>0.459484038967159</v>
+        <v>0.4691790858548</v>
       </c>
       <c r="O76" t="s">
         <v>20</v>
@@ -37829,7 +37829,7 @@
         <v>247</v>
       </c>
       <c r="N80" t="n">
-        <v>0.16150722981051</v>
+        <v>0.180960294529738</v>
       </c>
       <c r="O80" t="s">
         <v>26</v>
@@ -38033,7 +38033,7 @@
         <v>247</v>
       </c>
       <c r="N84" t="n">
-        <v>0.12796159934441</v>
+        <v>0.137562189816131</v>
       </c>
       <c r="O84" t="s">
         <v>42</v>
@@ -38190,7 +38190,7 @@
         <v>247</v>
       </c>
       <c r="N87" t="n">
-        <v>0.0726194425324379</v>
+        <v>0.0821885475321845</v>
       </c>
       <c r="O87" t="s">
         <v>38</v>
@@ -38243,7 +38243,7 @@
         <v>247</v>
       </c>
       <c r="N88" t="n">
-        <v>0.205642469943682</v>
+        <v>0.224938107303042</v>
       </c>
       <c r="O88" t="s">
         <v>26</v>
@@ -38296,7 +38296,7 @@
         <v>247</v>
       </c>
       <c r="N89" t="n">
-        <v>0.103433899047543</v>
+        <v>0.113191916879131</v>
       </c>
       <c r="O89" t="s">
         <v>42</v>
@@ -38400,7 +38400,7 @@
         <v>247</v>
       </c>
       <c r="N91" t="n">
-        <v>0.169397150998561</v>
+        <v>0.171550884495578</v>
       </c>
       <c r="O91" t="s">
         <v>26</v>
@@ -38506,7 +38506,7 @@
         <v>247</v>
       </c>
       <c r="N93" t="n">
-        <v>0.300427036016602</v>
+        <v>0.309964655544375</v>
       </c>
       <c r="O93" t="s">
         <v>20</v>
@@ -38559,7 +38559,7 @@
         <v>247</v>
       </c>
       <c r="N94" t="n">
-        <v>0.166855984985389</v>
+        <v>0.188084957537952</v>
       </c>
       <c r="O94" t="s">
         <v>26</v>
@@ -38612,7 +38612,7 @@
         <v>247</v>
       </c>
       <c r="N95" t="n">
-        <v>0.210820139484092</v>
+        <v>0.230115776843453</v>
       </c>
       <c r="O95" t="s">
         <v>26</v>
@@ -38665,7 +38665,7 @@
         <v>247</v>
       </c>
       <c r="N96" t="n">
-        <v>0.234557393536879</v>
+        <v>0.244283925896493</v>
       </c>
       <c r="O96" t="s">
         <v>26</v>
@@ -38716,7 +38716,7 @@
         <v>247</v>
       </c>
       <c r="N97" t="n">
-        <v>0.281096535433485</v>
+        <v>0.292819373930249</v>
       </c>
       <c r="O97" t="s">
         <v>20</v>
@@ -38767,7 +38767,7 @@
         <v>247</v>
       </c>
       <c r="N98" t="n">
-        <v>0.120135254463613</v>
+        <v>0.12228898796063</v>
       </c>
       <c r="O98" t="s">
         <v>42</v>
@@ -38820,7 +38820,7 @@
         <v>247</v>
       </c>
       <c r="N99" t="n">
-        <v>0.168480957760984</v>
+        <v>0.180172310785774</v>
       </c>
       <c r="O99" t="s">
         <v>26</v>
@@ -39187,7 +39187,7 @@
         <v>247</v>
       </c>
       <c r="N106" t="n">
-        <v>0.219774235157993</v>
+        <v>0.22192796865501</v>
       </c>
       <c r="O106" t="s">
         <v>26</v>
@@ -39344,7 +39344,7 @@
         <v>247</v>
       </c>
       <c r="N109" t="n">
-        <v>0.134678893267576</v>
+        <v>0.144216512795349</v>
       </c>
       <c r="O109" t="s">
         <v>42</v>
@@ -39446,7 +39446,7 @@
         <v>247</v>
       </c>
       <c r="N111" t="n">
-        <v>0.494017711023271</v>
+        <v>0.503712757910912</v>
       </c>
       <c r="O111" t="s">
         <v>20</v>
@@ -39497,7 +39497,7 @@
         <v>247</v>
       </c>
       <c r="N112" t="n">
-        <v>0.487011326660829</v>
+        <v>0.496580431660575</v>
       </c>
       <c r="O112" t="s">
         <v>20</v>
@@ -39650,7 +39650,7 @@
         <v>247</v>
       </c>
       <c r="N115" t="n">
-        <v>0.527882205570981</v>
+        <v>0.537419825098754</v>
       </c>
       <c r="O115" t="s">
         <v>20</v>
@@ -39701,7 +39701,7 @@
         <v>247</v>
       </c>
       <c r="N116" t="n">
-        <v>0.115521367102578</v>
+        <v>0.125090472102325</v>
       </c>
       <c r="O116" t="s">
         <v>42</v>
@@ -39803,7 +39803,7 @@
         <v>247</v>
       </c>
       <c r="N118" t="n">
-        <v>0.487997175368161</v>
+        <v>0.497818164143696</v>
       </c>
       <c r="O118" t="s">
         <v>20</v>
@@ -39905,7 +39905,7 @@
         <v>247</v>
       </c>
       <c r="N120" t="n">
-        <v>0.449491822586785</v>
+        <v>0.459060927586531</v>
       </c>
       <c r="O120" t="s">
         <v>20</v>
@@ -40415,7 +40415,7 @@
         <v>247</v>
       </c>
       <c r="N130" t="n">
-        <v>0.122854010946783</v>
+        <v>0.120700277449766</v>
       </c>
       <c r="O130" t="s">
         <v>42</v>
@@ -40925,7 +40925,7 @@
         <v>247</v>
       </c>
       <c r="N140" t="n">
-        <v>0.361533486617351</v>
+        <v>0.371071106145124</v>
       </c>
       <c r="O140" t="s">
         <v>20</v>
@@ -41082,7 +41082,7 @@
         <v>247</v>
       </c>
       <c r="N143" t="n">
-        <v>0.292783367877424</v>
+        <v>0.290629634380407</v>
       </c>
       <c r="O143" t="s">
         <v>20</v>
@@ -41135,13 +41135,13 @@
         <v>247</v>
       </c>
       <c r="N144" t="n">
-        <v>0.263080445909677</v>
+        <v>0.270779186660168</v>
       </c>
       <c r="O144" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="P144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q144" t="s">
         <v>246</v>
@@ -41188,7 +41188,7 @@
         <v>247</v>
       </c>
       <c r="N145" t="n">
-        <v>0.479358486470311</v>
+        <v>0.488896105998084</v>
       </c>
       <c r="O145" t="s">
         <v>20</v>
@@ -41239,7 +41239,7 @@
         <v>247</v>
       </c>
       <c r="N146" t="n">
-        <v>0.0531135567313678</v>
+        <v>0.0509598232343507</v>
       </c>
       <c r="O146" t="s">
         <v>38</v>
@@ -41557,7 +41557,7 @@
         <v>247</v>
       </c>
       <c r="N152" t="n">
-        <v>0.20301455242334</v>
+        <v>0.21261514289506</v>
       </c>
       <c r="O152" t="s">
         <v>26</v>
@@ -41663,7 +41663,7 @@
         <v>247</v>
       </c>
       <c r="N154" t="n">
-        <v>0.254177629082527</v>
+        <v>0.263746734082273</v>
       </c>
       <c r="O154" t="s">
         <v>26</v>
@@ -41716,13 +41716,13 @@
         <v>247</v>
       </c>
       <c r="N155" t="n">
-        <v>0.157734541137433</v>
+        <v>0.167335131609153</v>
       </c>
       <c r="O155" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="P155" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q155" t="s">
         <v>246</v>
@@ -42246,7 +42246,7 @@
         <v>247</v>
       </c>
       <c r="N165" t="n">
-        <v>0.43319261674325</v>
+        <v>0.442761721742997</v>
       </c>
       <c r="O165" t="s">
         <v>20</v>
@@ -42352,7 +42352,7 @@
         <v>247</v>
       </c>
       <c r="N167" t="n">
-        <v>0.39029885569023</v>
+        <v>0.399930931633923</v>
       </c>
       <c r="O167" t="s">
         <v>20</v>
@@ -42927,7 +42927,7 @@
         <v>247</v>
       </c>
       <c r="N178" t="n">
-        <v>0.136619161311979</v>
+        <v>0.134465427814962</v>
       </c>
       <c r="O178" t="s">
         <v>42</v>
@@ -43192,7 +43192,7 @@
         <v>247</v>
       </c>
       <c r="N183" t="n">
-        <v>0.0730837646485635</v>
+        <v>0.0829047534240982</v>
       </c>
       <c r="O183" t="s">
         <v>38</v>
@@ -43243,7 +43243,7 @@
         <v>247</v>
       </c>
       <c r="N184" t="n">
-        <v>0.0226195294797795</v>
+        <v>0.0322830908954467</v>
       </c>
       <c r="O184" t="s">
         <v>38</v>
@@ -43296,7 +43296,7 @@
         <v>247</v>
       </c>
       <c r="N185" t="n">
-        <v>0.196949864271371</v>
+        <v>0.194796130774354</v>
       </c>
       <c r="O185" t="s">
         <v>26</v>
@@ -43349,13 +43349,13 @@
         <v>247</v>
       </c>
       <c r="N186" t="n">
-        <v>0.260698192464484</v>
+        <v>0.279962344351872</v>
       </c>
       <c r="O186" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="P186" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q186" t="s">
         <v>246</v>
@@ -43402,7 +43402,7 @@
         <v>247</v>
       </c>
       <c r="N187" t="n">
-        <v>0.0329514326659267</v>
+        <v>0.0352625935228114</v>
       </c>
       <c r="O187" t="s">
         <v>38</v>
@@ -43504,7 +43504,7 @@
         <v>247</v>
       </c>
       <c r="N189" t="n">
-        <v>0.164921554686205</v>
+        <v>0.167075288183222</v>
       </c>
       <c r="O189" t="s">
         <v>26</v>
@@ -43555,7 +43555,7 @@
         <v>247</v>
       </c>
       <c r="N190" t="n">
-        <v>0.273619846142505</v>
+        <v>0.283314893030146</v>
       </c>
       <c r="O190" t="s">
         <v>20</v>
@@ -43657,7 +43657,7 @@
         <v>247</v>
       </c>
       <c r="N192" t="n">
-        <v>0.764539944366864</v>
+        <v>0.774077563894637</v>
       </c>
       <c r="O192" t="s">
         <v>20</v>
@@ -43761,7 +43761,7 @@
         <v>247</v>
       </c>
       <c r="N194" t="n">
-        <v>0.241933469829401</v>
+        <v>0.251534060301121</v>
       </c>
       <c r="O194" t="s">
         <v>26</v>
@@ -43814,7 +43814,7 @@
         <v>247</v>
       </c>
       <c r="N195" t="n">
-        <v>0.162603715092841</v>
+        <v>0.181962323396149</v>
       </c>
       <c r="O195" t="s">
         <v>26</v>
@@ -43867,7 +43867,7 @@
         <v>247</v>
       </c>
       <c r="N196" t="n">
-        <v>0.314848107062628</v>
+        <v>0.312694373565611</v>
       </c>
       <c r="O196" t="s">
         <v>20</v>
@@ -44026,7 +44026,7 @@
         <v>247</v>
       </c>
       <c r="N199" t="n">
-        <v>0.127915860268404</v>
+        <v>0.137453479796177</v>
       </c>
       <c r="O199" t="s">
         <v>42</v>
@@ -56017,10 +56017,10 @@
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
@@ -56029,7 +56029,7 @@
         <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
         <v>3</v>
@@ -56616,7 +56616,7 @@
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
         <v>2</v>
@@ -59154,7 +59154,7 @@
         <v>2</v>
       </c>
       <c r="G78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H78" t="n">
         <v>2</v>
@@ -62386,7 +62386,7 @@
         <v>42</v>
       </c>
       <c r="F131" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G131" t="n">
         <v>2</v>
@@ -62743,7 +62743,7 @@
         <v>2</v>
       </c>
       <c r="G137" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H137" t="n">
         <v>2</v>
@@ -63053,7 +63053,7 @@
         <v>2</v>
       </c>
       <c r="H142" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I142" t="n">
         <v>3</v>
@@ -63180,7 +63180,7 @@
         <v>2</v>
       </c>
       <c r="G144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H144" t="n">
         <v>4</v>
@@ -63762,7 +63762,7 @@
         <v>2</v>
       </c>
       <c r="H153" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I153" t="n">
         <v>1</v>
@@ -63880,13 +63880,13 @@
         <v>1</v>
       </c>
       <c r="D155" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E155" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="F155" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G155" t="n">
         <v>2</v>
@@ -65745,7 +65745,7 @@
         <v>2</v>
       </c>
       <c r="H184" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I184" t="n">
         <v>3</v>
@@ -65987,7 +65987,7 @@
         <v>26</v>
       </c>
       <c r="F188" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G188" t="n">
         <v>2</v>

</xml_diff>